<commit_message>
new day to day bank statement comparison
</commit_message>
<xml_diff>
--- a/comparativo_de_caixa.xlsx
+++ b/comparativo_de_caixa.xlsx
@@ -8,20 +8,21 @@
   </bookViews>
   <sheets>
     <sheet name="Resultados Gerais" sheetId="1" r:id="rId1"/>
-    <sheet name="caixa" sheetId="2" r:id="rId2"/>
-    <sheet name="cora_unidade_1_e_2" sheetId="3" r:id="rId3"/>
-    <sheet name="cora_unidade_3" sheetId="4" r:id="rId4"/>
-    <sheet name="itau_unidade_1_e_2" sheetId="5" r:id="rId5"/>
-    <sheet name="itau_unidade_3" sheetId="6" r:id="rId6"/>
-    <sheet name="sicredi_unidade_1_e_2" sheetId="7" r:id="rId7"/>
-    <sheet name="sicredi_unidade_3" sheetId="8" r:id="rId8"/>
+    <sheet name="Consolidado Diário" sheetId="2" r:id="rId2"/>
+    <sheet name="caixa" sheetId="3" r:id="rId3"/>
+    <sheet name="cora_unidade_1_e_2" sheetId="4" r:id="rId4"/>
+    <sheet name="cora_unidade_3" sheetId="5" r:id="rId5"/>
+    <sheet name="itau_unidade_1_e_2" sheetId="6" r:id="rId6"/>
+    <sheet name="itau_unidade_3" sheetId="7" r:id="rId7"/>
+    <sheet name="sicredi_unidade_1_e_2" sheetId="8" r:id="rId8"/>
+    <sheet name="sicredi_unidade_3" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="309" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="55">
   <si>
     <t>Banco</t>
   </si>
@@ -74,6 +75,96 @@
     <t>TOTAL</t>
   </si>
   <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>Dif. Rec.</t>
+  </si>
+  <si>
+    <t>Dif. Pag.</t>
+  </si>
+  <si>
+    <t>2026-01-01</t>
+  </si>
+  <si>
+    <t>2026-01-02</t>
+  </si>
+  <si>
+    <t>2026-01-03</t>
+  </si>
+  <si>
+    <t>2026-01-05</t>
+  </si>
+  <si>
+    <t>2026-01-06</t>
+  </si>
+  <si>
+    <t>2026-01-07</t>
+  </si>
+  <si>
+    <t>2026-01-08</t>
+  </si>
+  <si>
+    <t>2026-01-09</t>
+  </si>
+  <si>
+    <t>2026-01-12</t>
+  </si>
+  <si>
+    <t>2026-01-13</t>
+  </si>
+  <si>
+    <t>2026-01-14</t>
+  </si>
+  <si>
+    <t>2026-01-15</t>
+  </si>
+  <si>
+    <t>2026-01-16</t>
+  </si>
+  <si>
+    <t>2026-01-17</t>
+  </si>
+  <si>
+    <t>2026-01-19</t>
+  </si>
+  <si>
+    <t>2026-01-20</t>
+  </si>
+  <si>
+    <t>2026-01-21</t>
+  </si>
+  <si>
+    <t>2026-01-22</t>
+  </si>
+  <si>
+    <t>2026-01-23</t>
+  </si>
+  <si>
+    <t>2026-01-24</t>
+  </si>
+  <si>
+    <t>2026-01-25</t>
+  </si>
+  <si>
+    <t>2026-01-26</t>
+  </si>
+  <si>
+    <t>2026-01-27</t>
+  </si>
+  <si>
+    <t>2026-01-28</t>
+  </si>
+  <si>
+    <t>2026-01-29</t>
+  </si>
+  <si>
+    <t>2026-01-30</t>
+  </si>
+  <si>
+    <t>2026-02-02</t>
+  </si>
+  <si>
     <t>date</t>
   </si>
   <si>
@@ -95,88 +186,7 @@
     <t>pagas_diff</t>
   </si>
   <si>
-    <t>2026-01-03</t>
-  </si>
-  <si>
-    <t>2026-01-05</t>
-  </si>
-  <si>
-    <t>2026-01-12</t>
-  </si>
-  <si>
-    <t>2026-01-19</t>
-  </si>
-  <si>
-    <t>2026-01-21</t>
-  </si>
-  <si>
-    <t>2026-01-27</t>
-  </si>
-  <si>
-    <t>2026-02-02</t>
-  </si>
-  <si>
     <t>soma</t>
-  </si>
-  <si>
-    <t>2026-01-02</t>
-  </si>
-  <si>
-    <t>2026-01-06</t>
-  </si>
-  <si>
-    <t>2026-01-07</t>
-  </si>
-  <si>
-    <t>2026-01-08</t>
-  </si>
-  <si>
-    <t>2026-01-09</t>
-  </si>
-  <si>
-    <t>2026-01-13</t>
-  </si>
-  <si>
-    <t>2026-01-14</t>
-  </si>
-  <si>
-    <t>2026-01-17</t>
-  </si>
-  <si>
-    <t>2026-01-20</t>
-  </si>
-  <si>
-    <t>2026-01-22</t>
-  </si>
-  <si>
-    <t>2026-01-25</t>
-  </si>
-  <si>
-    <t>2026-01-26</t>
-  </si>
-  <si>
-    <t>2026-01-28</t>
-  </si>
-  <si>
-    <t>2026-01-29</t>
-  </si>
-  <si>
-    <t>2026-01-30</t>
-  </si>
-  <si>
-    <t>2026-01-01</t>
-  </si>
-  <si>
-    <t>2026-01-15</t>
-  </si>
-  <si>
-    <t>2026-01-16</t>
-  </si>
-  <si>
-    <t>2026-01-23</t>
-  </si>
-  <si>
-    <t>2026-01-24</t>
   </si>
 </sst>
 </file>
@@ -286,7 +296,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -298,6 +308,8 @@
     <xf numFmtId="164" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -877,6 +889,864 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:I29"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="3" width="14.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="6" width="14.7109375" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" customWidth="1"/>
+    <col min="8" max="9" width="16.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9">
+      <c r="A1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="9">
+        <v>1633.82</v>
+      </c>
+      <c r="C2" s="9">
+        <v>0</v>
+      </c>
+      <c r="D2" s="10">
+        <v>1633.82</v>
+      </c>
+      <c r="E2" s="9">
+        <v>0</v>
+      </c>
+      <c r="F2" s="9">
+        <v>0</v>
+      </c>
+      <c r="G2" s="10">
+        <v>0</v>
+      </c>
+      <c r="H2" s="10">
+        <v>1633.82</v>
+      </c>
+      <c r="I2" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="9">
+        <v>2312.98</v>
+      </c>
+      <c r="C3" s="9">
+        <v>3853.84</v>
+      </c>
+      <c r="D3" s="10">
+        <v>-1540.86</v>
+      </c>
+      <c r="E3" s="9">
+        <v>0</v>
+      </c>
+      <c r="F3" s="9">
+        <v>0</v>
+      </c>
+      <c r="G3" s="10">
+        <v>0</v>
+      </c>
+      <c r="H3" s="10">
+        <v>2312.98</v>
+      </c>
+      <c r="I3" s="10">
+        <v>3853.84</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="9">
+        <v>0</v>
+      </c>
+      <c r="C4" s="9">
+        <v>6500</v>
+      </c>
+      <c r="D4" s="10">
+        <v>-6500</v>
+      </c>
+      <c r="E4" s="9">
+        <v>0</v>
+      </c>
+      <c r="F4" s="9">
+        <v>5596.28</v>
+      </c>
+      <c r="G4" s="10">
+        <v>-5596.28</v>
+      </c>
+      <c r="H4" s="10">
+        <v>0</v>
+      </c>
+      <c r="I4" s="10">
+        <v>903.72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="9">
+        <v>136597.74</v>
+      </c>
+      <c r="C5" s="9">
+        <v>138131.12</v>
+      </c>
+      <c r="D5" s="10">
+        <v>-1533.38</v>
+      </c>
+      <c r="E5" s="9">
+        <v>7304.18</v>
+      </c>
+      <c r="F5" s="9">
+        <v>68207.89999999999</v>
+      </c>
+      <c r="G5" s="10">
+        <v>-60903.72</v>
+      </c>
+      <c r="H5" s="10">
+        <v>129293.56</v>
+      </c>
+      <c r="I5" s="10">
+        <v>69923.22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="9">
+        <v>5144.6</v>
+      </c>
+      <c r="C6" s="9">
+        <v>5144.6</v>
+      </c>
+      <c r="D6" s="10">
+        <v>0</v>
+      </c>
+      <c r="E6" s="9">
+        <v>86148.41</v>
+      </c>
+      <c r="F6" s="9">
+        <v>86148.40999999999</v>
+      </c>
+      <c r="G6" s="10">
+        <v>0</v>
+      </c>
+      <c r="H6" s="10">
+        <v>-81003.81</v>
+      </c>
+      <c r="I6" s="10">
+        <v>-81003.81</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="9">
+        <v>718.88</v>
+      </c>
+      <c r="C7" s="9">
+        <v>21170.09</v>
+      </c>
+      <c r="D7" s="10">
+        <v>-20451.21</v>
+      </c>
+      <c r="E7" s="9">
+        <v>52163.18</v>
+      </c>
+      <c r="F7" s="9">
+        <v>52163.18</v>
+      </c>
+      <c r="G7" s="10">
+        <v>0</v>
+      </c>
+      <c r="H7" s="10">
+        <v>-51444.3</v>
+      </c>
+      <c r="I7" s="10">
+        <v>-30993.09</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="9">
+        <v>4648.940000000001</v>
+      </c>
+      <c r="C8" s="9">
+        <v>4419.3</v>
+      </c>
+      <c r="D8" s="10">
+        <v>229.64</v>
+      </c>
+      <c r="E8" s="9">
+        <v>4740.04</v>
+      </c>
+      <c r="F8" s="9">
+        <v>31740.04</v>
+      </c>
+      <c r="G8" s="10">
+        <v>-27000</v>
+      </c>
+      <c r="H8" s="10">
+        <v>-91.09999999999999</v>
+      </c>
+      <c r="I8" s="10">
+        <v>-27320.74</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="9">
+        <v>5630.809999999999</v>
+      </c>
+      <c r="C9" s="9">
+        <v>5975.37</v>
+      </c>
+      <c r="D9" s="10">
+        <v>-344.56</v>
+      </c>
+      <c r="E9" s="9">
+        <v>6176.98</v>
+      </c>
+      <c r="F9" s="9">
+        <v>6176.98</v>
+      </c>
+      <c r="G9" s="10">
+        <v>0</v>
+      </c>
+      <c r="H9" s="10">
+        <v>-546.17</v>
+      </c>
+      <c r="I9" s="10">
+        <v>-201.61</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B10" s="9">
+        <v>11731.13</v>
+      </c>
+      <c r="C10" s="9">
+        <v>11152.29</v>
+      </c>
+      <c r="D10" s="10">
+        <v>578.84</v>
+      </c>
+      <c r="E10" s="9">
+        <v>5819.06</v>
+      </c>
+      <c r="F10" s="9">
+        <v>5819.06</v>
+      </c>
+      <c r="G10" s="10">
+        <v>0</v>
+      </c>
+      <c r="H10" s="10">
+        <v>5912.07</v>
+      </c>
+      <c r="I10" s="10">
+        <v>5333.23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="9">
+        <v>24559.72</v>
+      </c>
+      <c r="C11" s="9">
+        <v>34553.54</v>
+      </c>
+      <c r="D11" s="10">
+        <v>-9993.82</v>
+      </c>
+      <c r="E11" s="9">
+        <v>1147.33</v>
+      </c>
+      <c r="F11" s="9">
+        <v>1147.33</v>
+      </c>
+      <c r="G11" s="10">
+        <v>0</v>
+      </c>
+      <c r="H11" s="10">
+        <v>23412.39</v>
+      </c>
+      <c r="I11" s="10">
+        <v>33406.21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="9">
+        <v>2634.98</v>
+      </c>
+      <c r="C12" s="9">
+        <v>2829.46</v>
+      </c>
+      <c r="D12" s="10">
+        <v>-194.48</v>
+      </c>
+      <c r="E12" s="9">
+        <v>12026.35</v>
+      </c>
+      <c r="F12" s="9">
+        <v>12026.35</v>
+      </c>
+      <c r="G12" s="10">
+        <v>0</v>
+      </c>
+      <c r="H12" s="10">
+        <v>-9391.370000000001</v>
+      </c>
+      <c r="I12" s="10">
+        <v>-9196.889999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="9">
+        <v>7658.82</v>
+      </c>
+      <c r="C13" s="9">
+        <v>8659.52</v>
+      </c>
+      <c r="D13" s="10">
+        <v>-1000.7</v>
+      </c>
+      <c r="E13" s="9">
+        <v>708.6400000000001</v>
+      </c>
+      <c r="F13" s="9">
+        <v>708.6400000000001</v>
+      </c>
+      <c r="G13" s="10">
+        <v>0</v>
+      </c>
+      <c r="H13" s="10">
+        <v>6950.18</v>
+      </c>
+      <c r="I13" s="10">
+        <v>7950.88</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="9">
+        <v>3670.45</v>
+      </c>
+      <c r="C14" s="9">
+        <v>3646.75</v>
+      </c>
+      <c r="D14" s="10">
+        <v>23.7</v>
+      </c>
+      <c r="E14" s="9">
+        <v>3897.45</v>
+      </c>
+      <c r="F14" s="9">
+        <v>3897.45</v>
+      </c>
+      <c r="G14" s="10">
+        <v>0</v>
+      </c>
+      <c r="H14" s="10">
+        <v>-227</v>
+      </c>
+      <c r="I14" s="10">
+        <v>-250.7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" s="9">
+        <v>0</v>
+      </c>
+      <c r="C15" s="9">
+        <v>0</v>
+      </c>
+      <c r="D15" s="10">
+        <v>0</v>
+      </c>
+      <c r="E15" s="9">
+        <v>25</v>
+      </c>
+      <c r="F15" s="9">
+        <v>25</v>
+      </c>
+      <c r="G15" s="10">
+        <v>0</v>
+      </c>
+      <c r="H15" s="10">
+        <v>-25</v>
+      </c>
+      <c r="I15" s="10">
+        <v>-25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" s="9">
+        <v>11693.81</v>
+      </c>
+      <c r="C16" s="9">
+        <v>11954.38</v>
+      </c>
+      <c r="D16" s="10">
+        <v>-260.57</v>
+      </c>
+      <c r="E16" s="9">
+        <v>1747.34</v>
+      </c>
+      <c r="F16" s="9">
+        <v>1747.34</v>
+      </c>
+      <c r="G16" s="10">
+        <v>0</v>
+      </c>
+      <c r="H16" s="10">
+        <v>9946.469999999999</v>
+      </c>
+      <c r="I16" s="10">
+        <v>10207.04</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B17" s="9">
+        <v>115589.7</v>
+      </c>
+      <c r="C17" s="9">
+        <v>115811.23</v>
+      </c>
+      <c r="D17" s="10">
+        <v>-221.53</v>
+      </c>
+      <c r="E17" s="9">
+        <v>99433.36</v>
+      </c>
+      <c r="F17" s="9">
+        <v>129433.36</v>
+      </c>
+      <c r="G17" s="10">
+        <v>-30000</v>
+      </c>
+      <c r="H17" s="10">
+        <v>16156.34</v>
+      </c>
+      <c r="I17" s="10">
+        <v>-13622.13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" s="9">
+        <v>4035.28</v>
+      </c>
+      <c r="C18" s="9">
+        <v>4003.96</v>
+      </c>
+      <c r="D18" s="10">
+        <v>31.32</v>
+      </c>
+      <c r="E18" s="9">
+        <v>10178.87</v>
+      </c>
+      <c r="F18" s="9">
+        <v>10178.87</v>
+      </c>
+      <c r="G18" s="10">
+        <v>0</v>
+      </c>
+      <c r="H18" s="10">
+        <v>-6143.59</v>
+      </c>
+      <c r="I18" s="10">
+        <v>-6174.91</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19" s="9">
+        <v>5053.530000000001</v>
+      </c>
+      <c r="C19" s="9">
+        <v>5035.38</v>
+      </c>
+      <c r="D19" s="10">
+        <v>18.15</v>
+      </c>
+      <c r="E19" s="9">
+        <v>0</v>
+      </c>
+      <c r="F19" s="9">
+        <v>0</v>
+      </c>
+      <c r="G19" s="10">
+        <v>0</v>
+      </c>
+      <c r="H19" s="10">
+        <v>5053.53</v>
+      </c>
+      <c r="I19" s="10">
+        <v>5035.38</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="9">
+        <v>1346.68</v>
+      </c>
+      <c r="C20" s="9">
+        <v>21353.22</v>
+      </c>
+      <c r="D20" s="10">
+        <v>-20006.54</v>
+      </c>
+      <c r="E20" s="9">
+        <v>5462.22</v>
+      </c>
+      <c r="F20" s="9">
+        <v>5462.22</v>
+      </c>
+      <c r="G20" s="10">
+        <v>0</v>
+      </c>
+      <c r="H20" s="10">
+        <v>-4115.54</v>
+      </c>
+      <c r="I20" s="10">
+        <v>15891</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21" s="9">
+        <v>258.54</v>
+      </c>
+      <c r="C21" s="9">
+        <v>0</v>
+      </c>
+      <c r="D21" s="10">
+        <v>258.54</v>
+      </c>
+      <c r="E21" s="9">
+        <v>0</v>
+      </c>
+      <c r="F21" s="9">
+        <v>0</v>
+      </c>
+      <c r="G21" s="10">
+        <v>0</v>
+      </c>
+      <c r="H21" s="10">
+        <v>258.54</v>
+      </c>
+      <c r="I21" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B22" s="9">
+        <v>603.75</v>
+      </c>
+      <c r="C22" s="9">
+        <v>603.75</v>
+      </c>
+      <c r="D22" s="10">
+        <v>0</v>
+      </c>
+      <c r="E22" s="9">
+        <v>0</v>
+      </c>
+      <c r="F22" s="9">
+        <v>0</v>
+      </c>
+      <c r="G22" s="10">
+        <v>0</v>
+      </c>
+      <c r="H22" s="10">
+        <v>603.75</v>
+      </c>
+      <c r="I22" s="10">
+        <v>603.75</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B23" s="9">
+        <v>4949.47</v>
+      </c>
+      <c r="C23" s="9">
+        <v>5017.44</v>
+      </c>
+      <c r="D23" s="10">
+        <v>-67.97</v>
+      </c>
+      <c r="E23" s="9">
+        <v>10472.59</v>
+      </c>
+      <c r="F23" s="9">
+        <v>10472.59</v>
+      </c>
+      <c r="G23" s="10">
+        <v>0</v>
+      </c>
+      <c r="H23" s="10">
+        <v>-5523.12</v>
+      </c>
+      <c r="I23" s="10">
+        <v>-5455.15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" s="9">
+        <v>16002.46</v>
+      </c>
+      <c r="C24" s="9">
+        <v>15513.76</v>
+      </c>
+      <c r="D24" s="10">
+        <v>488.7</v>
+      </c>
+      <c r="E24" s="9">
+        <v>1582.97</v>
+      </c>
+      <c r="F24" s="9">
+        <v>1582.97</v>
+      </c>
+      <c r="G24" s="10">
+        <v>0</v>
+      </c>
+      <c r="H24" s="10">
+        <v>14419.49</v>
+      </c>
+      <c r="I24" s="10">
+        <v>13930.79</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B25" s="9">
+        <v>3219.99</v>
+      </c>
+      <c r="C25" s="9">
+        <v>4582.54</v>
+      </c>
+      <c r="D25" s="10">
+        <v>-1362.55</v>
+      </c>
+      <c r="E25" s="9">
+        <v>1206.93</v>
+      </c>
+      <c r="F25" s="9">
+        <v>1206.93</v>
+      </c>
+      <c r="G25" s="10">
+        <v>0</v>
+      </c>
+      <c r="H25" s="10">
+        <v>2013.06</v>
+      </c>
+      <c r="I25" s="10">
+        <v>3375.61</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B26" s="9">
+        <v>4018.59</v>
+      </c>
+      <c r="C26" s="9">
+        <v>2588.04</v>
+      </c>
+      <c r="D26" s="10">
+        <v>1430.55</v>
+      </c>
+      <c r="E26" s="9">
+        <v>12166.49</v>
+      </c>
+      <c r="F26" s="9">
+        <v>12166.49</v>
+      </c>
+      <c r="G26" s="10">
+        <v>0</v>
+      </c>
+      <c r="H26" s="10">
+        <v>-8147.9</v>
+      </c>
+      <c r="I26" s="10">
+        <v>-9578.450000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B27" s="9">
+        <v>5414.53</v>
+      </c>
+      <c r="C27" s="9">
+        <v>5175.3</v>
+      </c>
+      <c r="D27" s="10">
+        <v>239.23</v>
+      </c>
+      <c r="E27" s="9">
+        <v>256</v>
+      </c>
+      <c r="F27" s="9">
+        <v>256</v>
+      </c>
+      <c r="G27" s="10">
+        <v>0</v>
+      </c>
+      <c r="H27" s="10">
+        <v>5158.53</v>
+      </c>
+      <c r="I27" s="10">
+        <v>4919.3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B28" s="9">
+        <v>0</v>
+      </c>
+      <c r="C28" s="9">
+        <v>740.12</v>
+      </c>
+      <c r="D28" s="10">
+        <v>-740.12</v>
+      </c>
+      <c r="E28" s="9">
+        <v>0</v>
+      </c>
+      <c r="F28" s="9">
+        <v>0</v>
+      </c>
+      <c r="G28" s="10">
+        <v>0</v>
+      </c>
+      <c r="H28" s="10">
+        <v>0</v>
+      </c>
+      <c r="I28" s="10">
+        <v>740.12</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B29" s="6">
+        <v>379129.2</v>
+      </c>
+      <c r="C29" s="6">
+        <v>438415</v>
+      </c>
+      <c r="D29" s="7">
+        <v>-59285.8</v>
+      </c>
+      <c r="E29" s="6">
+        <v>322663.39</v>
+      </c>
+      <c r="F29" s="6">
+        <v>446163.39</v>
+      </c>
+      <c r="G29" s="7">
+        <v>-123500</v>
+      </c>
+      <c r="H29" s="7">
+        <v>56465.81</v>
+      </c>
+      <c r="I29" s="7">
+        <v>-7748.39</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -890,30 +1760,30 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>23</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="8" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B2" s="8">
         <v>0</v>
@@ -936,7 +1806,7 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B3" s="8">
         <v>0</v>
@@ -959,7 +1829,7 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="8" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B4" s="8">
         <v>0</v>
@@ -982,7 +1852,7 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="8" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="B5" s="8">
         <v>0</v>
@@ -1005,7 +1875,7 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="8" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="B6" s="8">
         <v>0</v>
@@ -1028,7 +1898,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="8" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="B7" s="8">
         <v>0</v>
@@ -1051,7 +1921,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="8" t="s">
-        <v>30</v>
+        <v>46</v>
       </c>
       <c r="B8" s="8">
         <v>0</v>
@@ -1073,25 +1943,25 @@
       </c>
     </row>
     <row r="9" spans="1:7">
-      <c r="A9" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" s="9">
-        <v>0</v>
-      </c>
-      <c r="C9" s="9">
+      <c r="A9" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" s="11">
+        <v>0</v>
+      </c>
+      <c r="C9" s="11">
         <v>7240.12</v>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="12">
         <v>-7240.12</v>
       </c>
-      <c r="E9" s="9">
+      <c r="E9" s="11">
         <v>-8101.950000000001</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="11">
         <v>-8101.950000000001</v>
       </c>
-      <c r="G9" s="10">
+      <c r="G9" s="12">
         <v>0</v>
       </c>
     </row>
@@ -1100,7 +1970,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1116,30 +1986,30 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>23</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="8" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="B2" s="8">
         <v>476.4400000000001</v>
@@ -1162,7 +2032,7 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B3" s="8">
         <v>231.33</v>
@@ -1185,7 +2055,7 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="8" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="B4" s="8">
         <v>231.33</v>
@@ -1208,7 +2078,7 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="8" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="B5" s="8">
         <v>0</v>
@@ -1231,7 +2101,7 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="8" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="B6" s="8">
         <v>136.63</v>
@@ -1254,7 +2124,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="8" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B7" s="8">
         <v>1302.72</v>
@@ -1277,7 +2147,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="8" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B8" s="8">
         <v>918.5500000000001</v>
@@ -1300,7 +2170,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="8" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="B9" s="8">
         <v>408.15</v>
@@ -1323,7 +2193,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="8" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="B10" s="8">
         <v>150</v>
@@ -1346,7 +2216,7 @@
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="8" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B11" s="8">
         <v>0</v>
@@ -1369,7 +2239,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="8" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="B12" s="8">
         <v>101.01</v>
@@ -1392,7 +2262,7 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="8" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B13" s="8">
         <v>402.99</v>
@@ -1415,7 +2285,7 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="8" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="B14" s="8">
         <v>322.09</v>
@@ -1438,7 +2308,7 @@
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="8" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B15" s="8">
         <v>648.65</v>
@@ -1461,7 +2331,7 @@
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="8" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B16" s="8">
         <v>603.75</v>
@@ -1484,7 +2354,7 @@
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B17" s="8">
         <v>181.92</v>
@@ -1507,7 +2377,7 @@
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B18" s="8">
         <v>0</v>
@@ -1530,7 +2400,7 @@
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B19" s="8">
         <v>210</v>
@@ -1553,7 +2423,7 @@
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B20" s="8">
         <v>2091.62</v>
@@ -1575,25 +2445,25 @@
       </c>
     </row>
     <row r="21" spans="1:7">
-      <c r="A21" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B21" s="9">
+      <c r="A21" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B21" s="11">
         <v>8417.18</v>
       </c>
-      <c r="C21" s="9">
+      <c r="C21" s="11">
         <v>8417.18</v>
       </c>
-      <c r="D21" s="10">
-        <v>0</v>
-      </c>
-      <c r="E21" s="9">
+      <c r="D21" s="12">
+        <v>0</v>
+      </c>
+      <c r="E21" s="11">
         <v>-7231.8</v>
       </c>
-      <c r="F21" s="9">
+      <c r="F21" s="11">
         <v>-7231.8</v>
       </c>
-      <c r="G21" s="10">
+      <c r="G21" s="12">
         <v>0</v>
       </c>
     </row>
@@ -1602,7 +2472,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1618,30 +2488,30 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>23</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="8" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="B2" s="8">
         <v>0</v>
@@ -1664,7 +2534,7 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="8" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="B3" s="8">
         <v>163.71</v>
@@ -1687,7 +2557,7 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="8" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B4" s="8">
         <v>163.71</v>
@@ -1709,25 +2579,25 @@
       </c>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B5" s="9">
+      <c r="A5" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="11">
         <v>327.42</v>
       </c>
-      <c r="C5" s="9">
+      <c r="C5" s="11">
         <v>327.42</v>
       </c>
-      <c r="D5" s="10">
-        <v>0</v>
-      </c>
-      <c r="E5" s="9">
+      <c r="D5" s="12">
+        <v>0</v>
+      </c>
+      <c r="E5" s="11">
         <v>-60</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="11">
         <v>-60</v>
       </c>
-      <c r="G5" s="10">
+      <c r="G5" s="12">
         <v>0</v>
       </c>
     </row>
@@ -1736,7 +2606,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -1749,30 +2619,30 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>23</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="8" t="s">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="B2" s="8">
         <v>1578.12</v>
@@ -1795,7 +2665,7 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="8" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="B3" s="8">
         <v>1836.54</v>
@@ -1818,7 +2688,7 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B4" s="8">
         <v>106425.05</v>
@@ -1841,7 +2711,7 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="8" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="B5" s="8">
         <v>2498.76</v>
@@ -1864,7 +2734,7 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="8" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="B6" s="8">
         <v>718.87</v>
@@ -1887,7 +2757,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="8" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="B7" s="8">
         <v>1747.31</v>
@@ -1910,7 +2780,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="8" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B8" s="8">
         <v>368.99</v>
@@ -1933,7 +2803,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="8" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B9" s="8">
         <v>7381.33</v>
@@ -1956,7 +2826,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="8" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="B10" s="8">
         <v>17827.54</v>
@@ -1979,7 +2849,7 @@
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="8" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="B11" s="8">
         <v>346.47</v>
@@ -2002,7 +2872,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="8" t="s">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="B12" s="8">
         <v>6110.82</v>
@@ -2025,7 +2895,7 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="8" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="B13" s="8">
         <v>1140.38</v>
@@ -2048,7 +2918,7 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="8" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="B14" s="8">
         <v>7132.34</v>
@@ -2071,7 +2941,7 @@
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="8" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B15" s="8">
         <v>90367.62</v>
@@ -2094,7 +2964,7 @@
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="8" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="B16" s="8">
         <v>2313.54</v>
@@ -2117,7 +2987,7 @@
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="8" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B17" s="8">
         <v>1569.19</v>
@@ -2140,7 +3010,7 @@
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="8" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="B18" s="8">
         <v>606.5599999999999</v>
@@ -2163,7 +3033,7 @@
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="8" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="B19" s="8">
         <v>258.54</v>
@@ -2186,7 +3056,7 @@
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B20" s="8">
         <v>1512.76</v>
@@ -2209,7 +3079,7 @@
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="8" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="B21" s="8">
         <v>11423.28</v>
@@ -2232,7 +3102,7 @@
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B22" s="8">
         <v>1719.99</v>
@@ -2255,7 +3125,7 @@
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B23" s="8">
         <v>2937.74</v>
@@ -2278,7 +3148,7 @@
     </row>
     <row r="24" spans="1:7">
       <c r="A24" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B24" s="8">
         <v>1366.66</v>
@@ -2300,25 +3170,25 @@
       </c>
     </row>
     <row r="25" spans="1:7">
-      <c r="A25" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B25" s="9">
+      <c r="A25" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B25" s="11">
         <v>269188.4</v>
       </c>
-      <c r="C25" s="9">
+      <c r="C25" s="11">
         <v>301290.7999999999</v>
       </c>
-      <c r="D25" s="10">
+      <c r="D25" s="12">
         <v>-32102.4</v>
       </c>
-      <c r="E25" s="9">
+      <c r="E25" s="11">
         <v>-257547.49</v>
       </c>
-      <c r="F25" s="9">
+      <c r="F25" s="11">
         <v>-316047.4899999999</v>
       </c>
-      <c r="G25" s="10">
+      <c r="G25" s="12">
         <v>58500</v>
       </c>
     </row>
@@ -2327,7 +3197,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2342,30 +3212,30 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>23</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B2" s="8">
         <v>29941.36</v>
@@ -2388,7 +3258,7 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="8" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="B3" s="8">
         <v>2414.51</v>
@@ -2411,7 +3281,7 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="8" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="B4" s="8">
         <v>0.01</v>
@@ -2434,7 +3304,7 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="8" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="B5" s="8">
         <v>0</v>
@@ -2457,7 +3327,7 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="8" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B6" s="8">
         <v>0.02</v>
@@ -2480,7 +3350,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="8" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B7" s="8">
         <v>0.01</v>
@@ -2503,7 +3373,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="8" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="B8" s="8">
         <v>1440</v>
@@ -2526,7 +3396,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="8" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="B9" s="8">
         <v>0</v>
@@ -2549,7 +3419,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="8" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B10" s="8">
         <v>22485.71</v>
@@ -2572,7 +3442,7 @@
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B11" s="8">
         <v>0.04</v>
@@ -2595,7 +3465,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="8" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="B12" s="8">
         <v>4579.18</v>
@@ -2618,7 +3488,7 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B13" s="8">
         <v>0.1</v>
@@ -2640,25 +3510,25 @@
       </c>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B14" s="9">
+      <c r="A14" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B14" s="11">
         <v>60860.94</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="11">
         <v>80860.94</v>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="12">
         <v>-20000</v>
       </c>
-      <c r="E14" s="9">
+      <c r="E14" s="11">
         <v>-42482.71</v>
       </c>
-      <c r="F14" s="9">
+      <c r="F14" s="11">
         <v>-80482.71000000001</v>
       </c>
-      <c r="G14" s="10">
+      <c r="G14" s="12">
         <v>38000</v>
       </c>
     </row>
@@ -2667,7 +3537,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -2683,30 +3553,30 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>23</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="8" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="B2" s="8">
         <v>0</v>
@@ -2729,7 +3599,7 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="8" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="B3" s="8">
         <v>0</v>
@@ -2752,7 +3622,7 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="8" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B4" s="8">
         <v>3959.08</v>
@@ -2775,7 +3645,7 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="8" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B5" s="8">
         <v>3431.24</v>
@@ -2798,7 +3668,7 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="8" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="B6" s="8">
         <v>3017.66</v>
@@ -2821,7 +3691,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="8" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="B7" s="8">
         <v>272.1</v>
@@ -2844,7 +3714,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="8" t="s">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="B8" s="8">
         <v>1548</v>
@@ -2867,7 +3737,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="8" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="B9" s="8">
         <v>2490.16</v>
@@ -2890,7 +3760,7 @@
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="8" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="B10" s="8">
         <v>4460.46</v>
@@ -2913,7 +3783,7 @@
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="8" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B11" s="8">
         <v>2333.38</v>
@@ -2936,7 +3806,7 @@
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="8" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="B12" s="8">
         <v>1235.94</v>
@@ -2959,7 +3829,7 @@
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="8" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B13" s="8">
         <v>838.13</v>
@@ -2982,7 +3852,7 @@
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="8" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="B14" s="8">
         <v>740.12</v>
@@ -3005,7 +3875,7 @@
     </row>
     <row r="15" spans="1:7">
       <c r="A15" s="8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B15" s="8">
         <v>3101.93</v>
@@ -3028,7 +3898,7 @@
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="8" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="B16" s="8">
         <v>0</v>
@@ -3051,7 +3921,7 @@
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B17" s="8">
         <v>1500</v>
@@ -3074,7 +3944,7 @@
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B18" s="8">
         <v>870.75</v>
@@ -3097,7 +3967,7 @@
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B19" s="8">
         <v>1956.25</v>
@@ -3119,25 +3989,25 @@
       </c>
     </row>
     <row r="20" spans="1:7">
-      <c r="A20" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B20" s="9">
+      <c r="A20" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" s="11">
         <v>31755.2</v>
       </c>
-      <c r="C20" s="9">
+      <c r="C20" s="11">
         <v>31755.2</v>
       </c>
-      <c r="D20" s="10">
-        <v>0</v>
-      </c>
-      <c r="E20" s="9">
+      <c r="D20" s="12">
+        <v>0</v>
+      </c>
+      <c r="E20" s="11">
         <v>-7189.44</v>
       </c>
-      <c r="F20" s="9">
+      <c r="F20" s="11">
         <v>-25189.44</v>
       </c>
-      <c r="G20" s="10">
+      <c r="G20" s="12">
         <v>18000</v>
       </c>
     </row>
@@ -3146,7 +4016,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3161,30 +4031,30 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>22</v>
+        <v>52</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>23</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="8" t="s">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="B2" s="8">
         <v>55.7</v>
@@ -3207,7 +4077,7 @@
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="8" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="B3" s="8">
         <v>2765</v>
@@ -3230,7 +4100,7 @@
     </row>
     <row r="4" spans="1:7">
       <c r="A4" s="8" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="B4" s="8">
         <v>1866.37</v>
@@ -3253,7 +4123,7 @@
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="8" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="B5" s="8">
         <v>1866.41</v>
@@ -3276,7 +4146,7 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="8" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="B6" s="8">
         <v>39.91</v>
@@ -3299,7 +4169,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="8" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B7" s="8">
         <v>1833.85</v>
@@ -3322,7 +4192,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B8" s="8">
         <v>152.82</v>
@@ -3345,7 +4215,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="8" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="B9" s="8">
         <v>0</v>
@@ -3367,25 +4237,25 @@
       </c>
     </row>
     <row r="10" spans="1:7">
-      <c r="A10" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B10" s="9">
+      <c r="A10" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" s="11">
         <v>8580.059999999999</v>
       </c>
-      <c r="C10" s="9">
+      <c r="C10" s="11">
         <v>8523.34</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="12">
         <v>56.72</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="11">
         <v>-50</v>
       </c>
-      <c r="F10" s="9">
+      <c r="F10" s="11">
         <v>-9050</v>
       </c>
-      <c r="G10" s="10">
+      <c r="G10" s="12">
         <v>9000</v>
       </c>
     </row>

</xml_diff>